<commit_message>
Grow alcohol and tobacco quantities with the OBR's clearances per head
The importer now reads the OBR's tobacco clearances (Table 4.11) and
alcohol clearance forecasts (Table 4.12) and writes six per-head series
under gov.economic_assumptions.yoy_growth.obr.per_capita, one per product
group: clearance growth over one plus ons.population growth, to six
decimals. Dataset projection grows household weights by ons.population,
so weighted quantities grow with the clearances. Each quantity input
declares its group's index and is mapped to its series in
uprating_indices.yaml. The real-table fixtures gain the clearance sheets,
with each kept sheet's XML and the shared strings unchanged.

Fixes #2596.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/policyengine_uk/tests/fixtures/obr_receipts/obr_efo_march_2025_receipts.xlsx
+++ b/policyengine_uk/tests/fixtures/obr_receipts/obr_efo_march_2025_receipts.xlsx
@@ -17,6 +17,8 @@
     <ns0:sheet name="3.2" sheetId="194" ns7:id="rId4"/>
     <ns0:sheet name="3.7" sheetId="204" ns7:id="rId9"/>
     <ns0:sheet name="3.9" sheetId="192" ns7:id="rId11"/>
+    <ns0:sheet name="3.11" sheetId="208" ns7:id="rId13"/>
+    <ns0:sheet name="3.12" sheetId="209" ns7:id="rId14"/>
   </ns0:sheets>
   <ns0:definedNames>
     <ns0:definedName name="________tab3" localSheetId="20">!#REF!</ns0:definedName>
@@ -10413,6 +10415,1206 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FD633EC-985A-453A-B0BD-4801B0D465F1}">
+  <sheetPr codeName="Sheet13">
+    <tabColor theme="6"/>
+  </sheetPr>
+  <dimension ref="A1:K32"/>
+  <sheetFormatPr defaultColWidth="9.453125" defaultRowHeight="13"/>
+  <cols>
+    <col min="1" max="1" width="9.453125" style="29" customWidth="1"/>
+    <col min="2" max="2" width="31.453125" style="29" customWidth="1"/>
+    <col min="3" max="9" width="10" style="29" customWidth="1"/>
+    <col min="10" max="16384" width="9.453125" style="29"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="33.75" customHeight="1" thickBot="1">
+      <c r="A1" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="B1" s="17"/>
+      <c r="K1" s="227"/>
+    </row>
+    <row r="2" spans="1:11" ht="19.5" customHeight="1" thickBot="1">
+      <c r="B2" s="596" t="s">
+        <v>162</v>
+      </c>
+      <c r="C2" s="597"/>
+      <c r="D2" s="597"/>
+      <c r="E2" s="597"/>
+      <c r="F2" s="597"/>
+      <c r="G2" s="597"/>
+      <c r="H2" s="597"/>
+      <c r="I2" s="598"/>
+    </row>
+    <row r="3" spans="1:11" ht="13.5" customHeight="1">
+      <c r="B3" s="229"/>
+      <c r="C3" s="164" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" s="610" t="s">
+        <v>4</v>
+      </c>
+      <c r="E3" s="610"/>
+      <c r="F3" s="610"/>
+      <c r="G3" s="610"/>
+      <c r="H3" s="610"/>
+      <c r="I3" s="611"/>
+    </row>
+    <row r="4" spans="1:11" ht="13.5" customHeight="1">
+      <c r="B4" s="230"/>
+      <c r="C4" s="40" t="s">
+        <v>72</v>
+      </c>
+      <c r="D4" s="40" t="s">
+        <v>77</v>
+      </c>
+      <c r="E4" s="40" t="s">
+        <v>80</v>
+      </c>
+      <c r="F4" s="41" t="s">
+        <v>83</v>
+      </c>
+      <c r="G4" s="41" t="s">
+        <v>87</v>
+      </c>
+      <c r="H4" s="41" t="s">
+        <v>135</v>
+      </c>
+      <c r="I4" s="42" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="13.5" customHeight="1">
+      <c r="B5" s="231" t="s">
+        <v>140</v>
+      </c>
+      <c r="C5" s="232">
+        <v>15627.731050470811</v>
+      </c>
+      <c r="D5" s="232">
+        <v>12261.041140089925</v>
+      </c>
+      <c r="E5" s="232">
+        <v>11438.1506269399</v>
+      </c>
+      <c r="F5" s="232">
+        <v>10771.444927263899</v>
+      </c>
+      <c r="G5" s="232">
+        <v>9755.6604635170606</v>
+      </c>
+      <c r="H5" s="232">
+        <v>9050.0632507213813</v>
+      </c>
+      <c r="I5" s="233">
+        <v>8433.644038661012</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="13.5" customHeight="1">
+      <c r="B6" s="234" t="s">
+        <v>144</v>
+      </c>
+      <c r="C6" s="232">
+        <v>6366.8488877159707</v>
+      </c>
+      <c r="D6" s="232">
+        <v>5477.578299079556</v>
+      </c>
+      <c r="E6" s="232">
+        <v>5110.3924391171995</v>
+      </c>
+      <c r="F6" s="232">
+        <v>4804.1163790399869</v>
+      </c>
+      <c r="G6" s="232">
+        <v>4710.4282371139898</v>
+      </c>
+      <c r="H6" s="232">
+        <v>4929.9575164259941</v>
+      </c>
+      <c r="I6" s="233">
+        <v>4997.552643798188</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="13.5" customHeight="1">
+      <c r="B7" s="235" t="s">
+        <v>115</v>
+      </c>
+      <c r="C7" s="232"/>
+      <c r="D7" s="232"/>
+      <c r="E7" s="232"/>
+      <c r="F7" s="232"/>
+      <c r="G7" s="232"/>
+      <c r="H7" s="232"/>
+      <c r="I7" s="233"/>
+    </row>
+    <row r="8" spans="1:11" ht="13.5" customHeight="1">
+      <c r="B8" s="236" t="s">
+        <v>116</v>
+      </c>
+      <c r="C8" s="232">
+        <v>5644.9079149009858</v>
+      </c>
+      <c r="D8" s="232">
+        <v>4825.5065340171341</v>
+      </c>
+      <c r="E8" s="232">
+        <v>4479.7648617864206</v>
+      </c>
+      <c r="F8" s="232">
+        <v>4214.1485404444147</v>
+      </c>
+      <c r="G8" s="232">
+        <v>4129.9055352228661</v>
+      </c>
+      <c r="H8" s="232">
+        <v>4300.8386745465641</v>
+      </c>
+      <c r="I8" s="233">
+        <v>4358.7575896231874</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="13.5" customHeight="1" thickBot="1">
+      <c r="B9" s="237" t="s">
+        <v>117</v>
+      </c>
+      <c r="C9" s="238">
+        <v>721.94097281498466</v>
+      </c>
+      <c r="D9" s="238">
+        <v>652.07176506242217</v>
+      </c>
+      <c r="E9" s="238">
+        <v>630.62757733077865</v>
+      </c>
+      <c r="F9" s="238">
+        <v>589.96783859557229</v>
+      </c>
+      <c r="G9" s="238">
+        <v>580.52270189112392</v>
+      </c>
+      <c r="H9" s="238">
+        <v>629.11884187942985</v>
+      </c>
+      <c r="I9" s="239">
+        <v>638.79505417500013</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11">
+      <c r="B10" s="96"/>
+      <c r="C10" s="232"/>
+      <c r="D10" s="232"/>
+      <c r="E10" s="232"/>
+      <c r="F10" s="232"/>
+      <c r="G10" s="232"/>
+      <c r="H10" s="232"/>
+      <c r="I10" s="232"/>
+    </row>
+    <row r="25" spans="3:9">
+      <c r="C25" s="232"/>
+      <c r="D25" s="232"/>
+      <c r="E25" s="232"/>
+      <c r="F25" s="232"/>
+      <c r="G25" s="232"/>
+      <c r="H25" s="232"/>
+      <c r="I25" s="232"/>
+    </row>
+    <row r="26" spans="3:9">
+      <c r="C26" s="232"/>
+      <c r="D26" s="232"/>
+      <c r="E26" s="232"/>
+      <c r="F26" s="232"/>
+      <c r="G26" s="232"/>
+      <c r="H26" s="232"/>
+    </row>
+    <row r="27" spans="3:9">
+      <c r="C27" s="232"/>
+      <c r="D27" s="232"/>
+      <c r="E27" s="232"/>
+      <c r="F27" s="232"/>
+      <c r="G27" s="232"/>
+      <c r="H27" s="232"/>
+    </row>
+    <row r="28" spans="3:9">
+      <c r="C28" s="232"/>
+      <c r="D28" s="232"/>
+      <c r="E28" s="232"/>
+      <c r="F28" s="232"/>
+      <c r="G28" s="232"/>
+      <c r="H28" s="232"/>
+    </row>
+    <row r="31" spans="3:9">
+      <c r="C31" s="193"/>
+      <c r="D31" s="193"/>
+      <c r="E31" s="193"/>
+      <c r="F31" s="193"/>
+      <c r="G31" s="193"/>
+      <c r="H31" s="193"/>
+    </row>
+    <row r="32" spans="3:9">
+      <c r="C32" s="240"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="D3:I3"/>
+  </mergeCells>
+  <phoneticPr fontId="39" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="A1" location="Contents!A1" display="Back to contents" xr:uid="{F640A598-9E5A-4835-9386-045783020007}"/>
+  </hyperlinks>
+  <pageMargins left="0.74803149606299213" right="0.74803149606299213" top="0.98425196850393704" bottom="0.98425196850393704" header="0.51181102362204722" footer="0.51181102362204722"/>
+  <pageSetup paperSize="9" scale="82" orientation="landscape" r:id="rId1"/>
+  <headerFooter alignWithMargins="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3957F9A-7C4D-409C-A28F-BE8B87961F74}">
+  <sheetPr codeName="Sheet14">
+    <tabColor theme="6"/>
+  </sheetPr>
+  <dimension ref="A1:R60"/>
+  <sheetFormatPr defaultColWidth="9.453125" defaultRowHeight="13"/>
+  <cols>
+    <col min="1" max="1" width="9.453125" style="29" customWidth="1"/>
+    <col min="2" max="2" width="23.54296875" style="29" customWidth="1"/>
+    <col min="3" max="3" width="13" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="9" width="9.453125" style="29" customWidth="1"/>
+    <col min="10" max="16384" width="9.453125" style="29"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18" ht="33.75" customHeight="1" thickBot="1">
+      <c r="A1" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="K1" s="227"/>
+    </row>
+    <row r="2" spans="1:18" ht="19.5" customHeight="1" thickBot="1">
+      <c r="B2" s="620" t="s">
+        <v>163</v>
+      </c>
+      <c r="C2" s="621"/>
+      <c r="D2" s="621"/>
+      <c r="E2" s="621"/>
+      <c r="F2" s="621"/>
+      <c r="G2" s="621"/>
+      <c r="H2" s="621"/>
+      <c r="I2" s="622"/>
+    </row>
+    <row r="3" spans="1:18" ht="15.5">
+      <c r="B3" s="241"/>
+      <c r="C3" s="164" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" s="578" t="s">
+        <v>4</v>
+      </c>
+      <c r="E3" s="578"/>
+      <c r="F3" s="578"/>
+      <c r="G3" s="578"/>
+      <c r="H3" s="578"/>
+      <c r="I3" s="579"/>
+    </row>
+    <row r="4" spans="1:18">
+      <c r="B4" s="242"/>
+      <c r="C4" s="40" t="s">
+        <v>72</v>
+      </c>
+      <c r="D4" s="40" t="s">
+        <v>77</v>
+      </c>
+      <c r="E4" s="40" t="s">
+        <v>80</v>
+      </c>
+      <c r="F4" s="41" t="s">
+        <v>83</v>
+      </c>
+      <c r="G4" s="41" t="s">
+        <v>87</v>
+      </c>
+      <c r="H4" s="41" t="s">
+        <v>135</v>
+      </c>
+      <c r="I4" s="42" t="s">
+        <v>180</v>
+      </c>
+      <c r="L4" s="318"/>
+      <c r="M4" s="318"/>
+      <c r="N4" s="318"/>
+      <c r="O4" s="318"/>
+      <c r="P4" s="318"/>
+      <c r="Q4" s="318"/>
+      <c r="R4" s="318"/>
+    </row>
+    <row r="5" spans="1:18">
+      <c r="B5" s="150" t="s">
+        <v>118</v>
+      </c>
+      <c r="C5" s="243">
+        <v>2187.4517020691928</v>
+      </c>
+      <c r="D5" s="243">
+        <v>2126.8350107574711</v>
+      </c>
+      <c r="E5" s="243">
+        <v>2070.2709736807733</v>
+      </c>
+      <c r="F5" s="243">
+        <v>2095.6238816933683</v>
+      </c>
+      <c r="G5" s="243">
+        <v>2120.8081243011748</v>
+      </c>
+      <c r="H5" s="243">
+        <v>2150.5327548235268</v>
+      </c>
+      <c r="I5" s="244">
+        <v>2186.272795659931</v>
+      </c>
+      <c r="L5" s="318"/>
+      <c r="M5" s="318"/>
+      <c r="N5" s="318"/>
+      <c r="O5" s="318"/>
+      <c r="P5" s="318"/>
+      <c r="Q5" s="318"/>
+      <c r="R5" s="318"/>
+    </row>
+    <row r="6" spans="1:18">
+      <c r="B6" s="150" t="s">
+        <v>119</v>
+      </c>
+      <c r="C6" s="243">
+        <v>1621.636249677927</v>
+      </c>
+      <c r="D6" s="243">
+        <v>1573.6441470568238</v>
+      </c>
+      <c r="E6" s="243">
+        <v>1607.0439468571697</v>
+      </c>
+      <c r="F6" s="243">
+        <v>1610.5239097536778</v>
+      </c>
+      <c r="G6" s="243">
+        <v>1613.7824539108412</v>
+      </c>
+      <c r="H6" s="243">
+        <v>1619.4224366478315</v>
+      </c>
+      <c r="I6" s="244">
+        <v>1628.3315903069531</v>
+      </c>
+      <c r="L6" s="318"/>
+      <c r="M6" s="318"/>
+      <c r="N6" s="318"/>
+      <c r="O6" s="318"/>
+      <c r="P6" s="318"/>
+      <c r="Q6" s="318"/>
+      <c r="R6" s="318"/>
+    </row>
+    <row r="7" spans="1:18" ht="13.5" customHeight="1">
+      <c r="B7" s="325" t="s">
+        <v>204</v>
+      </c>
+      <c r="C7" s="245">
+        <v>1340.1037428613899</v>
+      </c>
+      <c r="D7" s="245">
+        <v>1312.0535264985322</v>
+      </c>
+      <c r="E7" s="245">
+        <v>1389.9011605254505</v>
+      </c>
+      <c r="F7" s="245">
+        <v>1434.1708714260512</v>
+      </c>
+      <c r="G7" s="245">
+        <v>1479.4828716853963</v>
+      </c>
+      <c r="H7" s="245">
+        <v>1528.8225597242151</v>
+      </c>
+      <c r="I7" s="246">
+        <v>1583.0771465525686</v>
+      </c>
+      <c r="L7" s="318"/>
+      <c r="M7" s="318"/>
+      <c r="N7" s="318"/>
+      <c r="O7" s="318"/>
+      <c r="P7" s="318"/>
+      <c r="Q7" s="318"/>
+      <c r="R7" s="318"/>
+    </row>
+    <row r="8" spans="1:18" ht="12" customHeight="1">
+      <c r="B8" s="614" t="s">
+        <v>205</v>
+      </c>
+      <c r="C8" s="623"/>
+      <c r="D8" s="623"/>
+      <c r="E8" s="623"/>
+      <c r="F8" s="623"/>
+      <c r="G8" s="623"/>
+      <c r="H8" s="623"/>
+      <c r="I8" s="624"/>
+      <c r="L8" s="318"/>
+      <c r="M8" s="318"/>
+      <c r="N8" s="318"/>
+      <c r="O8" s="318"/>
+      <c r="P8" s="318"/>
+      <c r="Q8" s="318"/>
+      <c r="R8" s="318"/>
+    </row>
+    <row r="9" spans="1:18" ht="12" customHeight="1" thickBot="1">
+      <c r="B9" s="617" t="s">
+        <v>206</v>
+      </c>
+      <c r="C9" s="618"/>
+      <c r="D9" s="618"/>
+      <c r="E9" s="618"/>
+      <c r="F9" s="618"/>
+      <c r="G9" s="618"/>
+      <c r="H9" s="618"/>
+      <c r="I9" s="619"/>
+      <c r="L9" s="318"/>
+      <c r="M9" s="318"/>
+      <c r="N9" s="318"/>
+      <c r="O9" s="318"/>
+      <c r="P9" s="318"/>
+      <c r="Q9" s="318"/>
+      <c r="R9" s="318"/>
+    </row>
+    <row r="10" spans="1:18" ht="13.5" thickBot="1">
+      <c r="L10" s="318"/>
+      <c r="M10" s="318"/>
+      <c r="N10" s="318"/>
+      <c r="O10" s="318"/>
+      <c r="P10" s="318"/>
+      <c r="Q10" s="318"/>
+      <c r="R10" s="318"/>
+    </row>
+    <row r="11" spans="1:18" ht="19.5" customHeight="1" thickBot="1">
+      <c r="B11" s="620" t="s">
+        <v>164</v>
+      </c>
+      <c r="C11" s="621"/>
+      <c r="D11" s="621"/>
+      <c r="E11" s="621"/>
+      <c r="F11" s="621"/>
+      <c r="G11" s="621"/>
+      <c r="H11" s="621"/>
+      <c r="I11" s="622"/>
+      <c r="L11" s="318"/>
+      <c r="M11" s="318"/>
+      <c r="N11" s="318"/>
+      <c r="O11" s="318"/>
+      <c r="P11" s="318"/>
+      <c r="Q11" s="318"/>
+      <c r="R11" s="318"/>
+    </row>
+    <row r="12" spans="1:18" ht="18.75" customHeight="1">
+      <c r="B12" s="247"/>
+      <c r="C12" s="612" t="s">
+        <v>2</v>
+      </c>
+      <c r="D12" s="612"/>
+      <c r="E12" s="612"/>
+      <c r="F12" s="612"/>
+      <c r="G12" s="612"/>
+      <c r="H12" s="612"/>
+      <c r="I12" s="613"/>
+      <c r="L12" s="318"/>
+      <c r="M12" s="318"/>
+      <c r="N12" s="318"/>
+      <c r="O12" s="318"/>
+      <c r="P12" s="318"/>
+      <c r="Q12" s="318"/>
+      <c r="R12" s="318"/>
+    </row>
+    <row r="13" spans="1:18" ht="15" customHeight="1">
+      <c r="B13" s="241"/>
+      <c r="C13" s="164" t="s">
+        <v>3</v>
+      </c>
+      <c r="D13" s="578" t="s">
+        <v>4</v>
+      </c>
+      <c r="E13" s="578"/>
+      <c r="F13" s="578"/>
+      <c r="G13" s="578"/>
+      <c r="H13" s="578"/>
+      <c r="I13" s="579"/>
+      <c r="L13" s="318"/>
+      <c r="M13" s="318"/>
+      <c r="N13" s="318"/>
+      <c r="O13" s="318"/>
+      <c r="P13" s="318"/>
+      <c r="Q13" s="318"/>
+      <c r="R13" s="318"/>
+    </row>
+    <row r="14" spans="1:18" ht="14.25" customHeight="1">
+      <c r="B14" s="242"/>
+      <c r="C14" s="40" t="s">
+        <v>72</v>
+      </c>
+      <c r="D14" s="40" t="s">
+        <v>77</v>
+      </c>
+      <c r="E14" s="40" t="s">
+        <v>80</v>
+      </c>
+      <c r="F14" s="41" t="s">
+        <v>83</v>
+      </c>
+      <c r="G14" s="41" t="s">
+        <v>87</v>
+      </c>
+      <c r="H14" s="41" t="s">
+        <v>135</v>
+      </c>
+      <c r="I14" s="42" t="s">
+        <v>180</v>
+      </c>
+      <c r="L14" s="318"/>
+      <c r="M14" s="318"/>
+      <c r="N14" s="318"/>
+      <c r="O14" s="318"/>
+      <c r="P14" s="318"/>
+      <c r="Q14" s="318"/>
+      <c r="R14" s="319"/>
+    </row>
+    <row r="15" spans="1:18">
+      <c r="B15" s="150" t="s">
+        <v>118</v>
+      </c>
+      <c r="C15" s="248">
+        <v>3.8050000000000002</v>
+      </c>
+      <c r="D15" s="248">
+        <v>3.6870002282181029</v>
+      </c>
+      <c r="E15" s="248">
+        <v>3.8010145826287087</v>
+      </c>
+      <c r="F15" s="248">
+        <v>3.9771568532753183</v>
+      </c>
+      <c r="G15" s="248">
+        <v>4.1625127701196201</v>
+      </c>
+      <c r="H15" s="248">
+        <v>4.3588857194389909</v>
+      </c>
+      <c r="I15" s="249">
+        <v>4.5649701656510207</v>
+      </c>
+      <c r="L15" s="318"/>
+      <c r="M15" s="318"/>
+      <c r="N15" s="318"/>
+      <c r="O15" s="318"/>
+      <c r="P15" s="318"/>
+      <c r="Q15" s="318"/>
+      <c r="R15" s="319"/>
+    </row>
+    <row r="16" spans="1:18">
+      <c r="B16" s="150" t="s">
+        <v>119</v>
+      </c>
+      <c r="C16" s="248">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="D16" s="248">
+        <v>4.5659999999999998</v>
+      </c>
+      <c r="E16" s="248">
+        <v>4.7489999999999997</v>
+      </c>
+      <c r="F16" s="248">
+        <v>4.9059999999999997</v>
+      </c>
+      <c r="G16" s="248">
+        <v>5.0640000000000001</v>
+      </c>
+      <c r="H16" s="248">
+        <v>5.226</v>
+      </c>
+      <c r="I16" s="249">
+        <v>5.3979999999999997</v>
+      </c>
+      <c r="L16" s="318"/>
+      <c r="M16" s="318"/>
+      <c r="N16" s="318"/>
+      <c r="O16" s="318"/>
+      <c r="P16" s="318"/>
+      <c r="Q16" s="318"/>
+      <c r="R16" s="319"/>
+    </row>
+    <row r="17" spans="2:18">
+      <c r="B17" s="150" t="s">
+        <v>120</v>
+      </c>
+      <c r="C17" s="248">
+        <v>4.1100000000000003</v>
+      </c>
+      <c r="D17" s="248">
+        <v>4.1619999999999999</v>
+      </c>
+      <c r="E17" s="248">
+        <v>4.4770000000000003</v>
+      </c>
+      <c r="F17" s="248">
+        <v>4.7699999999999996</v>
+      </c>
+      <c r="G17" s="248">
+        <v>5.069</v>
+      </c>
+      <c r="H17" s="248">
+        <v>5.3890000000000002</v>
+      </c>
+      <c r="I17" s="250">
+        <v>5.742</v>
+      </c>
+      <c r="L17" s="318"/>
+      <c r="M17" s="318"/>
+      <c r="N17" s="318"/>
+      <c r="O17" s="318"/>
+      <c r="P17" s="318"/>
+      <c r="Q17" s="318"/>
+      <c r="R17" s="319"/>
+    </row>
+    <row r="18" spans="2:18" ht="12" customHeight="1">
+      <c r="B18" s="614" t="s">
+        <v>55</v>
+      </c>
+      <c r="C18" s="615"/>
+      <c r="D18" s="615"/>
+      <c r="E18" s="615"/>
+      <c r="F18" s="615"/>
+      <c r="G18" s="615"/>
+      <c r="H18" s="615"/>
+      <c r="I18" s="616"/>
+      <c r="L18" s="318"/>
+      <c r="M18" s="318"/>
+      <c r="N18" s="318"/>
+      <c r="O18" s="318"/>
+      <c r="P18" s="318"/>
+      <c r="Q18" s="318"/>
+      <c r="R18" s="319"/>
+    </row>
+    <row r="19" spans="2:18" ht="12" customHeight="1" thickBot="1">
+      <c r="B19" s="617" t="s">
+        <v>206</v>
+      </c>
+      <c r="C19" s="618"/>
+      <c r="D19" s="618"/>
+      <c r="E19" s="618"/>
+      <c r="F19" s="618"/>
+      <c r="G19" s="618"/>
+      <c r="H19" s="618"/>
+      <c r="I19" s="619"/>
+      <c r="L19" s="318"/>
+      <c r="M19" s="318"/>
+      <c r="N19" s="318"/>
+      <c r="O19" s="318"/>
+      <c r="P19" s="318"/>
+      <c r="Q19" s="318"/>
+      <c r="R19" s="319"/>
+    </row>
+    <row r="22" spans="2:18">
+      <c r="B22" s="318"/>
+      <c r="C22" s="318"/>
+      <c r="D22" s="318"/>
+      <c r="E22" s="318"/>
+      <c r="F22" s="318"/>
+      <c r="G22" s="318"/>
+      <c r="H22" s="318"/>
+      <c r="I22" s="318"/>
+      <c r="J22" s="318"/>
+      <c r="K22" s="318"/>
+      <c r="L22" s="318"/>
+    </row>
+    <row r="23" spans="2:18">
+      <c r="B23" s="318"/>
+      <c r="C23" s="318"/>
+      <c r="D23" s="318"/>
+      <c r="E23" s="318"/>
+      <c r="F23" s="318"/>
+      <c r="G23" s="318"/>
+      <c r="H23" s="318"/>
+      <c r="I23" s="318"/>
+      <c r="J23" s="318"/>
+      <c r="K23" s="318"/>
+      <c r="L23" s="318"/>
+    </row>
+    <row r="24" spans="2:18" ht="19.399999999999999" customHeight="1">
+      <c r="B24" s="318"/>
+      <c r="C24" s="318"/>
+      <c r="D24" s="318"/>
+      <c r="E24" s="318"/>
+      <c r="F24" s="318"/>
+      <c r="G24" s="318"/>
+      <c r="H24" s="318"/>
+      <c r="I24" s="318"/>
+      <c r="J24" s="318"/>
+      <c r="K24" s="318"/>
+      <c r="L24" s="318"/>
+    </row>
+    <row r="25" spans="2:18" ht="19.399999999999999" customHeight="1">
+      <c r="B25" s="318"/>
+      <c r="C25" s="318"/>
+      <c r="D25" s="318"/>
+      <c r="E25" s="318"/>
+      <c r="F25" s="318"/>
+      <c r="G25" s="318"/>
+      <c r="H25" s="318"/>
+      <c r="I25" s="318"/>
+      <c r="J25" s="318"/>
+      <c r="K25" s="318"/>
+      <c r="L25" s="318"/>
+    </row>
+    <row r="26" spans="2:18">
+      <c r="B26" s="318"/>
+      <c r="C26" s="318"/>
+      <c r="D26" s="318"/>
+      <c r="E26" s="318"/>
+      <c r="F26" s="318"/>
+      <c r="G26" s="318"/>
+      <c r="H26" s="318"/>
+      <c r="I26" s="318"/>
+      <c r="J26" s="318"/>
+      <c r="K26" s="318"/>
+      <c r="L26" s="318"/>
+    </row>
+    <row r="27" spans="2:18">
+      <c r="B27" s="318"/>
+      <c r="C27" s="318"/>
+      <c r="D27" s="318"/>
+      <c r="E27" s="318"/>
+      <c r="F27" s="318"/>
+      <c r="G27" s="318"/>
+      <c r="H27" s="318"/>
+      <c r="I27" s="318"/>
+      <c r="J27" s="318"/>
+      <c r="K27" s="318"/>
+      <c r="L27" s="318"/>
+    </row>
+    <row r="28" spans="2:18">
+      <c r="B28" s="318"/>
+      <c r="C28" s="318"/>
+      <c r="D28" s="318"/>
+      <c r="E28" s="318"/>
+      <c r="F28" s="318"/>
+      <c r="G28" s="318"/>
+      <c r="H28" s="318"/>
+      <c r="I28" s="318"/>
+      <c r="J28" s="318"/>
+      <c r="K28" s="318"/>
+      <c r="L28" s="318"/>
+    </row>
+    <row r="29" spans="2:18">
+      <c r="B29" s="318"/>
+      <c r="C29" s="318"/>
+      <c r="D29" s="318"/>
+      <c r="E29" s="318"/>
+      <c r="F29" s="318"/>
+      <c r="G29" s="318"/>
+      <c r="H29" s="318"/>
+      <c r="I29" s="318"/>
+      <c r="J29" s="318"/>
+      <c r="K29" s="318"/>
+      <c r="L29" s="318"/>
+    </row>
+    <row r="30" spans="2:18">
+      <c r="B30" s="318"/>
+      <c r="C30" s="318"/>
+      <c r="D30" s="318"/>
+      <c r="E30" s="318"/>
+      <c r="F30" s="318"/>
+      <c r="G30" s="318"/>
+      <c r="H30" s="318"/>
+      <c r="I30" s="318"/>
+      <c r="J30" s="318"/>
+      <c r="K30" s="318"/>
+      <c r="L30" s="318"/>
+    </row>
+    <row r="31" spans="2:18">
+      <c r="B31" s="318"/>
+      <c r="C31" s="318"/>
+      <c r="D31" s="318"/>
+      <c r="E31" s="318"/>
+      <c r="F31" s="318"/>
+      <c r="G31" s="318"/>
+      <c r="H31" s="318"/>
+      <c r="I31" s="318"/>
+      <c r="J31" s="318"/>
+      <c r="K31" s="318"/>
+      <c r="L31" s="318"/>
+    </row>
+    <row r="32" spans="2:18">
+      <c r="B32" s="318"/>
+      <c r="C32" s="318"/>
+      <c r="D32" s="318"/>
+      <c r="E32" s="318"/>
+      <c r="F32" s="318"/>
+      <c r="G32" s="318"/>
+      <c r="H32" s="318"/>
+      <c r="I32" s="318"/>
+      <c r="J32" s="318"/>
+      <c r="K32" s="318"/>
+      <c r="L32" s="318"/>
+    </row>
+    <row r="33" spans="2:12" ht="18.649999999999999" customHeight="1">
+      <c r="B33" s="318"/>
+      <c r="C33" s="318"/>
+      <c r="D33" s="318"/>
+      <c r="E33" s="318"/>
+      <c r="F33" s="318"/>
+      <c r="G33" s="318"/>
+      <c r="H33" s="318"/>
+      <c r="I33" s="318"/>
+      <c r="J33" s="318"/>
+      <c r="K33" s="318"/>
+      <c r="L33" s="318"/>
+    </row>
+    <row r="34" spans="2:12" ht="19.399999999999999" customHeight="1">
+      <c r="B34" s="318"/>
+      <c r="C34" s="318"/>
+      <c r="D34" s="318"/>
+      <c r="E34" s="318"/>
+      <c r="F34" s="318"/>
+      <c r="G34" s="318"/>
+      <c r="H34" s="318"/>
+      <c r="I34" s="318"/>
+      <c r="J34" s="318"/>
+      <c r="K34" s="318"/>
+      <c r="L34" s="318"/>
+    </row>
+    <row r="35" spans="2:12">
+      <c r="B35" s="318"/>
+      <c r="C35" s="318"/>
+      <c r="D35" s="318"/>
+      <c r="E35" s="318"/>
+      <c r="F35" s="318"/>
+      <c r="G35" s="318"/>
+      <c r="H35" s="318"/>
+      <c r="I35" s="318"/>
+      <c r="J35" s="318"/>
+      <c r="K35" s="318"/>
+      <c r="L35" s="318"/>
+    </row>
+    <row r="36" spans="2:12">
+      <c r="B36" s="318"/>
+      <c r="C36" s="318"/>
+      <c r="D36" s="318"/>
+      <c r="E36" s="318"/>
+      <c r="F36" s="318"/>
+      <c r="G36" s="318"/>
+      <c r="H36" s="318"/>
+      <c r="I36" s="318"/>
+      <c r="J36" s="318"/>
+      <c r="K36" s="318"/>
+      <c r="L36" s="318"/>
+    </row>
+    <row r="37" spans="2:12">
+      <c r="B37" s="318"/>
+      <c r="C37" s="318"/>
+      <c r="D37" s="318"/>
+      <c r="E37" s="318"/>
+      <c r="F37" s="318"/>
+      <c r="G37" s="318"/>
+      <c r="H37" s="318"/>
+      <c r="I37" s="318"/>
+      <c r="J37" s="318"/>
+      <c r="K37" s="318"/>
+      <c r="L37" s="318"/>
+    </row>
+    <row r="38" spans="2:12">
+      <c r="B38" s="318"/>
+      <c r="C38" s="318"/>
+      <c r="D38" s="318"/>
+      <c r="E38" s="318"/>
+      <c r="F38" s="318"/>
+      <c r="G38" s="318"/>
+      <c r="H38" s="318"/>
+      <c r="I38" s="318"/>
+      <c r="J38" s="318"/>
+      <c r="K38" s="318"/>
+      <c r="L38" s="318"/>
+    </row>
+    <row r="39" spans="2:12">
+      <c r="B39" s="318"/>
+      <c r="C39" s="318"/>
+      <c r="D39" s="318"/>
+      <c r="E39" s="318"/>
+      <c r="F39" s="318"/>
+      <c r="G39" s="318"/>
+      <c r="H39" s="318"/>
+      <c r="I39" s="318"/>
+      <c r="J39" s="318"/>
+      <c r="K39" s="318"/>
+      <c r="L39" s="318"/>
+    </row>
+    <row r="40" spans="2:12">
+      <c r="B40" s="318"/>
+      <c r="C40" s="318"/>
+      <c r="D40" s="318"/>
+      <c r="E40" s="318"/>
+      <c r="F40" s="318"/>
+      <c r="G40" s="318"/>
+      <c r="H40" s="318"/>
+      <c r="I40" s="318"/>
+      <c r="J40" s="318"/>
+      <c r="K40" s="318"/>
+      <c r="L40" s="318"/>
+    </row>
+    <row r="41" spans="2:12">
+      <c r="B41" s="318"/>
+      <c r="C41" s="318"/>
+      <c r="D41" s="318"/>
+      <c r="E41" s="318"/>
+      <c r="F41" s="318"/>
+      <c r="G41" s="318"/>
+      <c r="H41" s="318"/>
+      <c r="I41" s="318"/>
+      <c r="J41" s="318"/>
+      <c r="K41" s="318"/>
+      <c r="L41" s="318"/>
+    </row>
+    <row r="42" spans="2:12">
+      <c r="B42" s="318"/>
+      <c r="C42" s="318"/>
+      <c r="D42" s="318"/>
+      <c r="E42" s="318"/>
+      <c r="F42" s="318"/>
+      <c r="G42" s="318"/>
+      <c r="H42" s="318"/>
+      <c r="I42" s="318"/>
+      <c r="J42" s="318"/>
+      <c r="K42" s="318"/>
+      <c r="L42" s="318"/>
+    </row>
+    <row r="43" spans="2:12">
+      <c r="B43" s="318"/>
+      <c r="C43" s="318"/>
+      <c r="D43" s="318"/>
+      <c r="E43" s="318"/>
+      <c r="F43" s="318"/>
+      <c r="G43" s="318"/>
+      <c r="H43" s="318"/>
+      <c r="I43" s="318"/>
+      <c r="J43" s="318"/>
+      <c r="K43" s="318"/>
+      <c r="L43" s="318"/>
+    </row>
+    <row r="44" spans="2:12">
+      <c r="B44" s="318"/>
+      <c r="C44" s="318"/>
+      <c r="D44" s="318"/>
+      <c r="E44" s="318"/>
+      <c r="F44" s="318"/>
+      <c r="G44" s="318"/>
+      <c r="H44" s="318"/>
+      <c r="I44" s="318"/>
+      <c r="J44" s="318"/>
+      <c r="K44" s="318"/>
+      <c r="L44" s="318"/>
+    </row>
+    <row r="45" spans="2:12">
+      <c r="B45" s="318"/>
+      <c r="C45" s="318"/>
+      <c r="D45" s="318"/>
+      <c r="E45" s="318"/>
+      <c r="F45" s="318"/>
+      <c r="G45" s="318"/>
+      <c r="H45" s="318"/>
+      <c r="I45" s="318"/>
+      <c r="J45" s="318"/>
+      <c r="K45" s="318"/>
+      <c r="L45" s="318"/>
+    </row>
+    <row r="46" spans="2:12">
+      <c r="B46" s="318"/>
+      <c r="C46" s="318"/>
+      <c r="D46" s="318"/>
+      <c r="E46" s="318"/>
+      <c r="F46" s="318"/>
+      <c r="G46" s="318"/>
+      <c r="H46" s="318"/>
+      <c r="I46" s="318"/>
+      <c r="J46" s="318"/>
+      <c r="K46" s="318"/>
+      <c r="L46" s="318"/>
+    </row>
+    <row r="47" spans="2:12">
+      <c r="B47" s="318"/>
+      <c r="C47" s="318"/>
+      <c r="D47" s="318"/>
+      <c r="E47" s="318"/>
+      <c r="F47" s="318"/>
+      <c r="G47" s="318"/>
+      <c r="H47" s="318"/>
+      <c r="I47" s="318"/>
+      <c r="J47" s="318"/>
+      <c r="K47" s="318"/>
+      <c r="L47" s="318"/>
+    </row>
+    <row r="48" spans="2:12">
+      <c r="B48" s="318"/>
+      <c r="C48" s="318"/>
+      <c r="D48" s="318"/>
+      <c r="E48" s="318"/>
+      <c r="F48" s="318"/>
+      <c r="G48" s="318"/>
+      <c r="H48" s="318"/>
+      <c r="I48" s="318"/>
+      <c r="J48" s="318"/>
+      <c r="K48" s="318"/>
+      <c r="L48" s="318"/>
+    </row>
+    <row r="49" spans="2:12">
+      <c r="B49" s="318"/>
+      <c r="C49" s="318"/>
+      <c r="D49" s="318"/>
+      <c r="E49" s="318"/>
+      <c r="F49" s="318"/>
+      <c r="G49" s="318"/>
+      <c r="H49" s="318"/>
+      <c r="I49" s="318"/>
+      <c r="J49" s="318"/>
+      <c r="K49" s="318"/>
+      <c r="L49" s="318"/>
+    </row>
+    <row r="50" spans="2:12">
+      <c r="B50" s="318"/>
+      <c r="C50" s="318"/>
+      <c r="D50" s="318"/>
+      <c r="E50" s="318"/>
+      <c r="F50" s="318"/>
+      <c r="G50" s="318"/>
+      <c r="H50" s="318"/>
+      <c r="I50" s="318"/>
+      <c r="J50" s="318"/>
+      <c r="K50" s="318"/>
+      <c r="L50" s="318"/>
+    </row>
+    <row r="51" spans="2:12">
+      <c r="B51" s="318"/>
+      <c r="C51" s="318"/>
+      <c r="D51" s="318"/>
+      <c r="E51" s="318"/>
+      <c r="F51" s="318"/>
+      <c r="G51" s="318"/>
+      <c r="H51" s="318"/>
+      <c r="I51" s="318"/>
+      <c r="J51" s="318"/>
+      <c r="K51" s="318"/>
+      <c r="L51" s="318"/>
+    </row>
+    <row r="52" spans="2:12">
+      <c r="B52" s="318"/>
+      <c r="C52" s="318"/>
+      <c r="D52" s="318"/>
+      <c r="E52" s="318"/>
+      <c r="F52" s="318"/>
+      <c r="G52" s="318"/>
+      <c r="H52" s="318"/>
+      <c r="I52" s="318"/>
+      <c r="J52" s="318"/>
+      <c r="K52" s="318"/>
+      <c r="L52" s="318"/>
+    </row>
+    <row r="53" spans="2:12">
+      <c r="B53" s="318"/>
+      <c r="C53" s="318"/>
+      <c r="D53" s="318"/>
+      <c r="E53" s="318"/>
+      <c r="F53" s="318"/>
+      <c r="G53" s="318"/>
+      <c r="H53" s="318"/>
+      <c r="I53" s="318"/>
+      <c r="J53" s="318"/>
+      <c r="K53" s="318"/>
+      <c r="L53" s="318"/>
+    </row>
+    <row r="54" spans="2:12">
+      <c r="B54" s="318"/>
+      <c r="C54" s="318"/>
+      <c r="D54" s="318"/>
+      <c r="E54" s="318"/>
+      <c r="F54" s="318"/>
+      <c r="G54" s="318"/>
+      <c r="H54" s="318"/>
+      <c r="I54" s="318"/>
+      <c r="J54" s="318"/>
+      <c r="K54" s="318"/>
+      <c r="L54" s="318"/>
+    </row>
+    <row r="55" spans="2:12">
+      <c r="B55" s="318"/>
+      <c r="C55" s="318"/>
+      <c r="D55" s="318"/>
+      <c r="E55" s="318"/>
+      <c r="F55" s="318"/>
+      <c r="G55" s="318"/>
+      <c r="H55" s="318"/>
+      <c r="I55" s="318"/>
+      <c r="J55" s="318"/>
+      <c r="K55" s="318"/>
+      <c r="L55" s="318"/>
+    </row>
+    <row r="56" spans="2:12">
+      <c r="B56" s="318"/>
+      <c r="C56" s="318"/>
+      <c r="D56" s="318"/>
+      <c r="E56" s="318"/>
+      <c r="F56" s="318"/>
+      <c r="G56" s="318"/>
+      <c r="H56" s="318"/>
+      <c r="I56" s="318"/>
+      <c r="J56" s="318"/>
+      <c r="K56" s="318"/>
+      <c r="L56" s="318"/>
+    </row>
+    <row r="57" spans="2:12">
+      <c r="B57" s="318"/>
+      <c r="C57" s="318"/>
+      <c r="D57" s="318"/>
+      <c r="E57" s="318"/>
+      <c r="F57" s="318"/>
+      <c r="G57" s="318"/>
+      <c r="H57" s="318"/>
+      <c r="I57" s="318"/>
+      <c r="J57" s="318"/>
+      <c r="K57" s="318"/>
+      <c r="L57" s="318"/>
+    </row>
+    <row r="60" spans="2:12">
+      <c r="B60" s="251"/>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="C12:I12"/>
+    <mergeCell ref="D13:I13"/>
+    <mergeCell ref="B18:I18"/>
+    <mergeCell ref="B19:I19"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="D3:I3"/>
+    <mergeCell ref="B8:I8"/>
+    <mergeCell ref="B9:I9"/>
+    <mergeCell ref="B11:I11"/>
+  </mergeCells>
+  <phoneticPr fontId="39" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="A1" location="Contents!A1" display="Back to contents" xr:uid="{9FA62B33-BAC6-4FD9-A12D-4178AF2CE126}"/>
+  </hyperlinks>
+  <pageMargins left="0.74803149606299213" right="0.74803149606299213" top="0.98425196850393704" bottom="0.98425196850393704" header="0.51181102362204722" footer="0.51181102362204722"/>
+  <pageSetup paperSize="9" scale="82" orientation="landscape" r:id="rId1"/>
+  <headerFooter alignWithMargins="0"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{657582D5-BD3B-4482-82A3-154823C755A5}">
   <sheetPr codeName="Sheet4">

</xml_diff>